<commit_message>
Add living-document link, per-document PDFs and complete compendium
- pdf/: business plan, deck, mind map, PM plan, tracker and meeting record
  as PDFs; 07_Complete_Compendium.pdf joins them all with bookmarks
- meeting/: summary and full transcript as received
- Content: smaller meeting details added so every output captures them;
  version 1.2 (21 Oct 2026); roadmap 'today' line driven by AS_OF
- Mind map embeds diagram PNGs so flowcharts render offline and in print
- Tracker gets A4 landscape print setup

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PuDfHj7dThQJ8wSqjxQQJi
</commit_message>
<xml_diff>
--- a/business-plans/prasadam-vertical/05_Project_Tracker.xlsx
+++ b/business-plans/prasadam-vertical/05_Project_Tracker.xlsx
@@ -27,7 +27,28 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open questions" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market research" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Read me'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'WBS &amp; Gantt'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'WBS &amp; Gantt'!$A$1:$K$50</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Milestones'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Action items'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'RACI'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Team &amp; roles'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Risk register'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Financial model'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Unit economics'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'KPI tracker'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'ROI &amp; hours log'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="11">'Revenue streams'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="12">'Audiences'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="13">'Products'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="14">'Gift tiers'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="15">'Festival calendar'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="16">'Business ideas'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="17">'Open questions'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="18">'Market research'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -616,7 +637,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -641,7 +662,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>v1.0 draft, 26 September 2026</t>
+          <t>v1.2, 21 October 2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +722,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -709,7 +740,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1171,7 +1202,17 @@
       <c r="Q11" s="27" t="n"/>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1179,7 +1220,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2324,7 +2365,17 @@
       <formula1>"R1,R2,R3,R4,R5,R6,R7,R8,R9,R10,R11,R12,R13,R14"</formula1>
     </dataValidation>
   </dataValidations>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -2332,7 +2383,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3054,7 +3105,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -3062,7 +3123,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3632,7 +3693,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -3640,7 +3711,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4358,7 +4429,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -4366,7 +4447,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4488,7 +4569,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -4496,7 +4587,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4898,7 +4989,17 @@
       <c r="G15" s="11" t="inlineStr"/>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -4906,7 +5007,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -5186,7 +5287,17 @@
       <c r="E17" s="11" t="inlineStr"/>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -5194,7 +5305,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -5318,7 +5429,17 @@
       <c r="D10" s="11" t="inlineStr"/>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -5326,7 +5447,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -5580,7 +5701,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -5588,7 +5719,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BM50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -18830,7 +18961,17 @@
       <formula1>"Not started,In progress,Blocked,Done"</formula1>
     </dataValidation>
   </dataValidations>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -18838,7 +18979,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -19052,7 +19193,17 @@
       <c r="D11" s="11" t="inlineStr"/>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -19060,7 +19211,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -19442,7 +19593,17 @@
       <c r="F13" s="11" t="inlineStr"/>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -19450,7 +19611,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -20085,7 +20246,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -20093,7 +20264,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -20308,7 +20479,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -20316,7 +20497,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -20904,7 +21085,17 @@
       <formula>8</formula>
     </cfRule>
   </conditionalFormatting>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -20912,7 +21103,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -21835,7 +22026,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -21843,7 +22044,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -22087,6 +22288,16 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;A · page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>